<commit_message>
Regroupe 1ère Pro Aristée avec 2nde Pro Aristée
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SjSsUvYfWg3LPV8sLWWofN
</commit_message>
<xml_diff>
--- a/Classement_Classes.xlsx
+++ b/Classement_Classes.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -790,31 +790,31 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>260</v>
+        <v>241</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>10 – 13 – 14 – 27 – 47 – 48 – 49 – 52</t>
+          <t>5 – 7 – 16 – 22 – 34 – 36 – 39 – 82</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>LUSSIEZ Baptiste, TEMPEZ Antoine, CAMUS Hugo, BOUTEILLER Nathan, BOURGOGNE Célestine, COURTOIS Luka, LEVERT Quentin, BRUNEEL Pierre-Vincent</t>
+          <t>ROUSSEL Vivien, LAVISSE Paul-Edouard, BRIANCHON Evan, DEGENNE Valentin, VICTORIA Paul, HADENGUE Alban, BONNEVAL Baptiste, LAFFINEUR Enzo</t>
         </is>
       </c>
     </row>
@@ -824,31 +824,31 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1, 2</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>8</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>308</v>
+        <v>260</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>5 – 7 – 16 – 22 – 34 – 39 – 82 – 103</t>
+          <t>10 – 13 – 14 – 27 – 47 – 48 – 49 – 52</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>ROUSSEL Vivien, LAVISSE Paul-Edouard, BRIANCHON Evan, DEGENNE Valentin, VICTORIA Paul, BONNEVAL Baptiste, LAFFINEUR Enzo, DINDIN Lorenzo</t>
+          <t>LUSSIEZ Baptiste, TEMPEZ Antoine, CAMUS Hugo, BOUTEILLER Nathan, BOURGOGNE Célestine, COURTOIS Luka, LEVERT Quentin, BRUNEEL Pierre-Vincent</t>
         </is>
       </c>
     </row>
@@ -1162,75 +1162,43 @@
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro Aristée</t>
+          <t>GDEA 2 Sco</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>36</v>
+        <v>585</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>16 – 79 – 100 – 125 – 132 – 133</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>HADENGUE Alban</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>GDEA 2 Sco</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>585</v>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>16 – 79 – 100 – 125 – 132 – 133</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
           <t>SERGEANT Mathéo, GREBERT Jules, GRIERE Pierre, RENARD Louis, CARON Cyprien, CARTON Evan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Calcul : pour chaque classe, on additionne les places obtenues par ses 8 meilleurs élèves dans leur course. Le plus petit total gagne.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Calcul : pour chaque classe, on additionne les places obtenues par ses 8 meilleurs élèves dans leur course. Le plus petit total gagne.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Les classes avec moins de 8 coureurs sont listées à la fin, sans rang. Les profs ne comptent pas.</t>
         </is>
@@ -1247,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1517,164 +1485,164 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro Aristée</t>
+          <t>Tale Pro</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>HADENGUE</t>
+          <t>LEMPEREUR</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Alban</t>
+          <t>Antoine</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>11:11</t>
+          <t>8:52</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Tale Pro</t>
+          <t>ACSE 1 Déméter</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>LEMPEREUR</t>
+          <t>CHEVALLIER</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Antoine</t>
+          <t>Louis</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>8:52</t>
+          <t>9:14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>ACSE 1 Déméter</t>
+          <t>ACSE 1 Sco</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>CHEVALLIER</t>
+          <t>CLAREBOUT</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Louis</t>
+          <t>Dorian</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>9:14</t>
+          <t>9:51</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>ACSE 1 Sco</t>
+          <t>Tale STAV</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>CLAREBOUT</t>
+          <t>MAGNIEZ</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Dorian</t>
+          <t>Alexis</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>9:51</t>
+          <t>9:52</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Tale STAV</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>MAGNIEZ</t>
+          <t>VALENTIN</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Alexis</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>9:52</t>
+          <t>9:53</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>ACSE 1 Cérès</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>VALENTIN</t>
+          <t>DUCATEZ</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Noé</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
@@ -1685,52 +1653,52 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>ACSE 1 Cérès</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>DUCATEZ</t>
+          <t>GOSSELIN</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Noé</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>9:53</t>
+          <t>10:14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>ACSE 2 Sco</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>GOSSELIN</t>
+          <t>GERARD</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
@@ -1741,138 +1709,110 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>ACSE 2 Sco</t>
+          <t>GDEA 2 Sco</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>GERARD</t>
+          <t>SERGEANT</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Mathéo</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>10:14</t>
+          <t>10:33</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>GDEA 2 Sco</t>
+          <t>Tale G</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>SERGEANT</t>
+          <t>BOGNY</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Mathéo</t>
+          <t>Ylenzo</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>11:23</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Tale G</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>BOGNY</t>
+          <t>DONNEZ</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Ylenzo</t>
+          <t>Nino</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>DONNEZ</t>
+          <t>DEROEUX</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Nino</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>4ème</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>DEROEUX</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Aaron</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1889,7 +1829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G160"/>
+  <dimension ref="A1:G159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3925,7 +3865,7 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B66" s="4" t="n">
@@ -3933,30 +3873,30 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>LUSSIEZ</t>
+          <t>ROUSSEL</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Vivien</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>9:40</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
@@ -3964,30 +3904,30 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>TEMPEZ</t>
+          <t>LAVISSE</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Antoine</t>
+          <t>Paul-Edouard</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>9:55</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B68" s="4" t="n">
@@ -3995,30 +3935,30 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>CAMUS</t>
+          <t>BRIANCHON</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="E68" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:27</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B69" s="4" t="n">
@@ -4026,30 +3966,30 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>BOUTEILLER</t>
+          <t>DEGENNE</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Valentin</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:46</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B70" s="4" t="n">
@@ -4057,30 +3997,30 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>BOURGOGNE</t>
+          <t>VICTORIA</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Célestine</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>11:06</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
@@ -4088,30 +4028,30 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>COURTOIS</t>
+          <t>HADENGUE</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Luka</t>
+          <t>Alban</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>13:27</t>
+          <t>11:11</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B72" s="4" t="n">
@@ -4119,30 +4059,30 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>LEVERT</t>
+          <t>BONNEVAL</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Quentin</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>11:40</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B73" s="4" t="n">
@@ -4150,30 +4090,30 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>BRUNEEL</t>
+          <t>LAFFINEUR</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>Pierre-Vincent</t>
+          <t>Enzo</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>52</v>
+        <v>82</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>14:02</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B74" s="4" t="n">
@@ -4181,30 +4121,30 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>ROUSSEL</t>
+          <t>LUSSIEZ</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Vivien</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>10:01</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B75" s="4" t="n">
@@ -4212,30 +4152,30 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>LAVISSE</t>
+          <t>TEMPEZ</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Paul-Edouard</t>
+          <t>Antoine</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>9:55</t>
+          <t>10:20</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B76" s="4" t="n">
@@ -4243,30 +4183,30 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>BRIANCHON</t>
+          <t>CAMUS</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Evan</t>
+          <t>Hugo</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:24</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B77" s="4" t="n">
@@ -4274,30 +4214,30 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>DEGENNE</t>
+          <t>BOUTEILLER</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Valentin</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>10:46</t>
+          <t>10:51</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B78" s="4" t="n">
@@ -4305,30 +4245,30 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>BOURGOGNE</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Célestine</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>12:14</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B79" s="4" t="n">
@@ -4336,30 +4276,30 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>BONNEVAL</t>
+          <t>COURTOIS</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Luka</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>13:27</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B80" s="4" t="n">
@@ -4367,30 +4307,30 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>LAFFINEUR</t>
+          <t>LEVERT</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Enzo</t>
+          <t>Quentin</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>12:21</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B81" s="4" t="n">
@@ -4398,23 +4338,23 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>DINDIN</t>
+          <t>BRUNEEL</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Lorenzo</t>
+          <t>Pierre-Vincent</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>103</v>
+        <v>52</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>12:38</t>
         </is>
       </c>
     </row>
@@ -6653,7 +6593,7 @@
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro Aristée</t>
+          <t>GDEA 2 Sco</t>
         </is>
       </c>
       <c r="B154" s="4" t="n">
@@ -6661,23 +6601,23 @@
       </c>
       <c r="C154" s="5" t="inlineStr">
         <is>
-          <t>HADENGUE</t>
+          <t>SERGEANT</t>
         </is>
       </c>
       <c r="D154" s="5" t="inlineStr">
         <is>
-          <t>Alban</t>
+          <t>Mathéo</t>
         </is>
       </c>
       <c r="E154" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F154" s="4" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="G154" s="4" t="inlineStr">
         <is>
-          <t>11:11</t>
+          <t>10:33</t>
         </is>
       </c>
     </row>
@@ -6688,27 +6628,27 @@
         </is>
       </c>
       <c r="B155" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>SERGEANT</t>
+          <t>GREBERT</t>
         </is>
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>Mathéo</t>
+          <t>Jules</t>
         </is>
       </c>
       <c r="E155" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F155" s="4" t="n">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="G155" s="4" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>15:14</t>
         </is>
       </c>
     </row>
@@ -6719,27 +6659,27 @@
         </is>
       </c>
       <c r="B156" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>GREBERT</t>
+          <t>GRIERE</t>
         </is>
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="E156" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F156" s="4" t="n">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
-          <t>15:14</t>
+          <t>16:44</t>
         </is>
       </c>
     </row>
@@ -6750,27 +6690,27 @@
         </is>
       </c>
       <c r="B157" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>GRIERE</t>
+          <t>RENARD</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Louis</t>
         </is>
       </c>
       <c r="E157" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F157" s="4" t="n">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="G157" s="4" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>17:53</t>
         </is>
       </c>
     </row>
@@ -6781,27 +6721,27 @@
         </is>
       </c>
       <c r="B158" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C158" s="5" t="inlineStr">
         <is>
-          <t>RENARD</t>
+          <t>CARON</t>
         </is>
       </c>
       <c r="D158" s="5" t="inlineStr">
         <is>
-          <t>Louis</t>
+          <t>Cyprien</t>
         </is>
       </c>
       <c r="E158" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="G158" s="4" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>18:15</t>
         </is>
       </c>
     </row>
@@ -6812,56 +6752,25 @@
         </is>
       </c>
       <c r="B159" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>CARON</t>
+          <t>CARTON</t>
         </is>
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>Cyprien</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="E159" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G159" s="4" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="5" t="inlineStr">
-        <is>
-          <t>GDEA 2 Sco</t>
-        </is>
-      </c>
-      <c r="B160" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C160" s="5" t="inlineStr">
-        <is>
-          <t>CARTON</t>
-        </is>
-      </c>
-      <c r="D160" s="5" t="inlineStr">
-        <is>
-          <t>Evan</t>
-        </is>
-      </c>
-      <c r="E160" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F160" s="4" t="n">
-        <v>133</v>
-      </c>
-      <c r="G160" s="4" t="inlineStr">
         <is>
           <t>18:26</t>
         </is>

</xml_diff>

<commit_message>
Classement des classes au temps moyen des 8 meilleurs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SjSsUvYfWg3LPV8sLWWofN
</commit_message>
<xml_diff>
--- a/Classement_Classes.xlsx
+++ b/Classement_Classes.xlsx
@@ -465,8 +465,8 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
     <col width="110" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -498,12 +498,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Total des places</t>
+          <t>Temps moyen (8 meilleurs)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Places des 8 meilleurs</t>
+          <t>Temps des 8 meilleurs</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -518,31 +518,33 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1, 2</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>56</v>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1 – 2 – 3 – 7 – 8 – 9 – 10 – 16</t>
+          <t>8:49 – 9:53 – 10:25 – 10:34 – 10:42 – 10:45 – 10:47 – 11:14</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>DONNEZ Nino, DEBUIRE Victor, ROCROY Ethan, HACCART Lucas, BOULET Léo, CARPENTIER Antonin, LEFEVRE COUPE Elora, PROBIN Tristan</t>
+          <t>GRONNIER Matéo, DUFRANNE Léopold, PIETRZAK Eden, BELLIARD Julien, LESAFFRE Lucas, DESCAMPS Baptiste, PIOLE Jean, CARON Jules</t>
         </is>
       </c>
     </row>
@@ -552,31 +554,33 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>80</v>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>4 – 5 – 6 – 11 – 12 – 13 – 14 – 15</t>
+          <t>9:56 – 9:57 – 10:12 – 10:31 – 10:48 – 10:53 – 10:56 – 11:05</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>DEROEUX Aaron, WYCKAERT Lucas, ROCHE Timothé, DEVAUCHELLE Tyméo, DESFRANCOIS Lucas, LAMOUR Hugo, ROUGEGREZ Mael, GELE Yanis</t>
+          <t>HERLEMONT Maxime, DREANO-LENGLET Nicolas, BRUNIAUX Timothé, DELABRE Florimond, CAUCHY Milan, LELEUX Baptiste, CLAY Gabriel, GUILBERT Gabriel</t>
         </is>
       </c>
     </row>
@@ -586,31 +590,33 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>145</v>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2 – 9 – 15 – 18 – 20 – 21 – 23 – 37</t>
+          <t>8:38 – 9:20 – 9:41 – 10:50 – 10:54 – 11:53 – 13:04 – 13:14</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>GRONNIER Matéo, DUFRANNE Léopold, PIETRZAK Eden, BELLIARD Julien, LESAFFRE Lucas, DESCAMPS Baptiste, PIOLE Jean, CARON Jules</t>
+          <t>BERTHE Charles, LAUR Benjamin, BONEL Arthur, DESSENNE Adrien, DUPONT Alexandre, LEIGNEL Jeanne, WINTREBERT Marion, DEGARDIN Luna</t>
         </is>
       </c>
     </row>
@@ -620,7 +626,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -629,22 +635,24 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>161</v>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>8 – 9 – 12 – 17 – 25 – 28 – 30 – 32</t>
+          <t>9:40 – 9:55 – 10:27 – 10:46 – 11:06 – 11:11 – 11:40 – 14:02</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>HERLEMONT Maxime, DREANO-LENGLET Nicolas, BRUNIAUX Timothé, DELABRE Florimond, CAUCHY Milan, LELEUX Baptiste, CLAY Gabriel, GUILBERT Gabriel</t>
+          <t>ROUSSEL Vivien, LAVISSE Paul-Edouard, BRIANCHON Evan, DEGENNE Valentin, VICTORIA Paul, HADENGUE Alban, BONNEVAL Baptiste, LAFFINEUR Enzo</t>
         </is>
       </c>
     </row>
@@ -668,12 +676,14 @@
       <c r="E6" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>192</v>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>3 – 8 – 18 – 21 – 23 – 38 – 40 – 41</t>
+          <t>9:51 – 9:53 – 10:59 – 11:22 – 11:23 – 12:41 – 12:47 – 12:54</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -688,12 +698,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1, 2</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -702,17 +712,19 @@
       <c r="E7" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>220</v>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>1 – 4 – 6 – 26 – 29 – 41 – 56 – 57</t>
+          <t>10:01 – 10:20 – 10:24 – 10:51 – 12:14 – 12:21 – 12:38 – 13:27</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>BERTHE Charles, LAUR Benjamin, BONEL Arthur, DESSENNE Adrien, DUPONT Alexandre, LEIGNEL Jeanne, WINTREBERT Marion, DEGARDIN Luna</t>
+          <t>LUSSIEZ Baptiste, TEMPEZ Antoine, CAMUS Hugo, BOUTEILLER Nathan, BOURGOGNE Célestine, LEVERT Quentin, BRUNEEL Pierre-Vincent, FOVEAU Paul</t>
         </is>
       </c>
     </row>
@@ -736,12 +748,14 @@
       <c r="E8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>224</v>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2 – 4 – 22 – 30 – 33 – 42 – 45 – 46</t>
+          <t>9:14 – 9:52 – 11:22 – 11:55 – 11:57 – 12:54 – 13:11 – 13:22</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -756,31 +770,33 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>238</v>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>6 – 7 – 25 – 34 – 36 – 39 – 44 – 47</t>
+          <t>8:53 – 11:01 – 11:46 – 11:56 – 12:06 – 12:20 – 12:49 – 13:16</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>VALENTIN Baptiste, GAGNON Gabriel, CORRE Maël, MERVEILLE Arthur, DUHAMEL Rémi, TOP Tédy, ELIE Quantin, DULOT Baptiste</t>
+          <t>BOURBON Raphael, LEIGNEL Madeline, DRUET Gabriel, BRULIN Albéric, LEMAITRE Lola, LETOURMY Maximilien, GROS Léopold, CUCHEVAL Mary</t>
         </is>
       </c>
     </row>
@@ -790,12 +806,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
@@ -804,17 +820,19 @@
       <c r="E10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>241</v>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>11:48</t>
+        </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>5 – 7 – 16 – 22 – 34 – 36 – 39 – 82</t>
+          <t>10:06 – 10:19 – 10:22 – 11:18 – 11:48 – 12:36 – 12:37 – 15:15</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>ROUSSEL Vivien, LAVISSE Paul-Edouard, BRIANCHON Evan, DEGENNE Valentin, VICTORIA Paul, HADENGUE Alban, BONNEVAL Baptiste, LAFFINEUR Enzo</t>
+          <t>DONNEZ Nino, DEBUIRE Victor, ROCROY Ethan, HACCART Lucas, BOULET Léo, CARPENTIER Antonin, LEFEVRE COUPE Elora, PROBIN Tristan</t>
         </is>
       </c>
     </row>
@@ -824,31 +842,33 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>260</v>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>10 – 13 – 14 – 27 – 47 – 48 – 49 – 52</t>
+          <t>9:53 – 9:53 – 11:23 – 11:58 – 12:31 – 12:41 – 13:00 – 13:22</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>LUSSIEZ Baptiste, TEMPEZ Antoine, CAMUS Hugo, BOUTEILLER Nathan, BOURGOGNE Célestine, COURTOIS Luka, LEVERT Quentin, BRUNEEL Pierre-Vincent</t>
+          <t>VALENTIN Baptiste, GAGNON Gabriel, CORRE Maël, MERVEILLE Arthur, DUHAMEL Rémi, TOP Tédy, ELIE Quantin, DULOT Baptiste</t>
         </is>
       </c>
     </row>
@@ -858,31 +878,33 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1, 2</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>322</v>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>3 – 31 – 40 – 42 – 46 – 48 – 54 – 58</t>
+          <t>10:04 – 10:32 – 11:08 – 12:29 – 13:00 – 13:59 – 13:59 – 14:00</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>BOURBON Raphael, LEIGNEL Madeline, DRUET Gabriel, BRULIN Albéric, LEMAITRE Lola, LETOURMY Maximilien, GROS Léopold, CUCHEVAL Mary</t>
+          <t>DUPONT Gabriel, VALCKE Anthime, LAMIAUX Paul, MILLE Lubin, POLIN Clémentine, VIARD Camille, COPIN Léontine, LAVAQUERIE Léa</t>
         </is>
       </c>
     </row>
@@ -906,12 +928,14 @@
       <c r="E13" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>356</v>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>1 – 17 – 35 – 37 – 52 – 61 – 75 – 78</t>
+          <t>8:52 – 10:58 – 12:21 – 12:41 – 13:43 – 14:15 – 15:05 – 15:05</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -940,12 +964,14 @@
       <c r="E14" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>367</v>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>12 – 19 – 27 – 29 – 31 – 80 – 81 – 88</t>
+          <t>10:14 – 10:59 – 11:24 – 11:39 – 11:56 – 15:18 – 15:29 – 16:05</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -974,12 +1000,14 @@
       <c r="E15" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F15" s="4" t="n">
-        <v>378</v>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>5 – 13 – 49 – 50 – 57 – 67 – 68 – 69</t>
+          <t>9:52 – 10:15 – 13:32 – 13:32 – 13:58 – 14:29 – 14:40 – 14:40</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -994,7 +1022,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1003,22 +1031,24 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F16" s="4" t="n">
-        <v>392</v>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>11 – 15 – 35 – 50 – 55 – 73 – 75 – 78</t>
+          <t>10:37 – 11:59 – 12:42 – 13:29 – 13:58 – 13:58 – 14:04 – 14:49</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>DUPONT Gabriel, VALCKE Anthime, LAMIAUX Paul, MILLE Lubin, POLIN Clémentine, VIARD Camille, COPIN Léontine, LAVAQUERIE Léa</t>
+          <t>DERUIT Maxime, ANSELIN Lucas, CAMUS Pierre, COMBLE Pierre, BERTOUX Jules, LAGACHE Mathieu, DALLERY Jules, VIGNE--PLAISANT Marius</t>
         </is>
       </c>
     </row>
@@ -1028,31 +1058,33 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>426</v>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>11 – 14 – 26 – 32 – 65 – 83 – 92 – 103</t>
+          <t>10:41 – 10:42 – 11:00 – 14:31 – 14:32 – 14:42 – 15:13 – 15:14</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>GOSSELIN Arthur, BELKHAYAT Thibaut, MINEZ Clément, DELVA Simon, GRIN Louis, GENCE Raphaël, SNEESSENS Gabriel, DELCROIX Alexis</t>
+          <t>DEROEUX Aaron, WYCKAERT Lucas, ROCHE Timothé, DEVAUCHELLE Tyméo, DESFRANCOIS Lucas, LAMOUR Hugo, ROUGEGREZ Mael, GELE Yanis</t>
         </is>
       </c>
     </row>
@@ -1062,12 +1094,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
@@ -1076,17 +1108,19 @@
       <c r="E18" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>450</v>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>19 – 43 – 53 – 58 – 67 – 69 – 70 – 71</t>
+          <t>10:14 – 10:31 – 11:24 – 11:57 – 14:21 – 15:49 – 16:16 – 16:54</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>DERUIT Maxime, ANSELIN Lucas, CAMUS Pierre, DALLERY Jules, COMBLE Pierre, BERTOUX Jules, VIGNE--PLAISANT Marius, LAGACHE Mathieu</t>
+          <t>GOSSELIN Arthur, BELKHAYAT Thibaut, MINEZ Clément, DELVA Simon, GRIN Louis, GENCE Raphaël, SNEESSENS Gabriel, DELCROIX Alexis</t>
         </is>
       </c>
     </row>
@@ -1110,12 +1144,14 @@
       <c r="E19" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F19" s="4" t="n">
-        <v>586</v>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>14:49</t>
+        </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>10 – 55 – 62 – 73 – 77 – 82 – 110 – 117</t>
+          <t>9:53 – 13:58 – 14:21 – 14:49 – 15:05 – 15:38 – 17:14 – 17:37</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1144,12 +1180,14 @@
       <c r="E20" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F20" s="4" t="n">
-        <v>871</v>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>24 – 28 – 84 – 114 – 131 – 145 – 157 – 188</t>
+          <t>11:23 – 11:34 – 15:49 – 17:18 – 18:05 – 19:02 – 19:31 – 21:01</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -1176,12 +1214,14 @@
       <c r="E21" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F21" s="4" t="n">
-        <v>585</v>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>16 – 79 – 100 – 125 – 132 – 133</t>
+          <t>10:33 – 15:14 – 16:44 – 17:53 – 18:15 – 18:26</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1193,14 +1233,14 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Calcul : pour chaque classe, on additionne les places obtenues par ses 8 meilleurs élèves dans leur course. Le plus petit total gagne.</t>
+          <t>Calcul : pour chaque classe, on fait la moyenne des temps de ses 8 élèves les plus rapides. Le plus petit temps moyen gagne.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Les classes avec moins de 8 coureurs sont listées à la fin, sans rang. Les profs ne comptent pas.</t>
+          <t>Les classes avec moins de 8 coureurs sont listées à la fin, sans rang (moyenne sur leurs coureurs). Les profs ne comptent pas.</t>
         </is>
       </c>
     </row>
@@ -1317,360 +1357,360 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>Tale Pro</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>BOURBON</t>
+          <t>LEMPEREUR</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Raphael</t>
+          <t>Antoine</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>8:53</t>
+          <t>8:52</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>ROUSSEL</t>
+          <t>BOURBON</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Vivien</t>
+          <t>Raphael</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>8:53</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>ACSE 1 Déméter</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>HERLEMONT</t>
+          <t>CHEVALLIER</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Maxime</t>
+          <t>Louis</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>9:56</t>
+          <t>9:14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>LUSSIEZ</t>
+          <t>ROUSSEL</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Vivien</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>9:40</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>ACSE 1 Sco</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>DUPONT</t>
+          <t>CLAREBOUT</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Dorian</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>9:51</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>Tale STAV</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>DERUIT</t>
+          <t>MAGNIEZ</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Maxime</t>
+          <t>Alexis</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>10:37</t>
+          <t>9:52</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Tale Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>LEMPEREUR</t>
+          <t>VALENTIN</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Antoine</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>8:52</t>
+          <t>9:53</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>ACSE 1 Déméter</t>
+          <t>ACSE 1 Cérès</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>CHEVALLIER</t>
+          <t>DUCATEZ</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Louis</t>
+          <t>Noé</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>9:14</t>
+          <t>9:53</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>ACSE 1 Sco</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>CLAREBOUT</t>
+          <t>HERLEMONT</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Dorian</t>
+          <t>Maxime</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>9:51</t>
+          <t>9:56</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Tale STAV</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>MAGNIEZ</t>
+          <t>LUSSIEZ</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Alexis</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>9:52</t>
+          <t>10:01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>VALENTIN</t>
+          <t>DUPONT</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>9:53</t>
+          <t>10:04</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>ACSE 1 Cérès</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>DUCATEZ</t>
+          <t>DONNEZ</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Noé</t>
+          <t>Nino</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>9:53</t>
+          <t>10:06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>ACSE 2 Sco</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>GOSSELIN</t>
+          <t>GERARD</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="D16" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
@@ -1681,24 +1721,24 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>ACSE 2 Sco</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>GERARD</t>
+          <t>GOSSELIN</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
@@ -1737,84 +1777,84 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Tale G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>BOGNY</t>
+          <t>DERUIT</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Ylenzo</t>
+          <t>Maxime</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>10:37</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>DONNEZ</t>
+          <t>DEROEUX</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Nino</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:41</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>Tale G</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>DEROEUX</t>
+          <t>BOGNY</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Ylenzo</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:23</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1921,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -1889,30 +1929,30 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>DONNEZ</t>
+          <t>GRONNIER</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Nino</t>
+          <t>Matéo</t>
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
@@ -1920,30 +1960,30 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>DEBUIRE</t>
+          <t>DUFRANNE</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Victor</t>
+          <t>Léopold</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9:53</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -1951,30 +1991,30 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ROCROY</t>
+          <t>PIETRZAK</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Ethan</t>
+          <t>Eden</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:25</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -1982,30 +2022,30 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>HACCART</t>
+          <t>BELLIARD</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Julien</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:34</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
@@ -2013,30 +2053,30 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BOULET</t>
+          <t>LESAFFRE</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Léo</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:42</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -2044,30 +2084,30 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>CARPENTIER</t>
+          <t>DESCAMPS</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Antonin</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:45</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -2075,30 +2115,30 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>LEFEVRE COUPE</t>
+          <t>PIOLE</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Elora</t>
+          <t>Jean</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:47</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>3ème</t>
+          <t>1ère STAV</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -2106,30 +2146,30 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>PROBIN</t>
+          <t>CARON</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Tristan</t>
+          <t>Jules</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -2137,30 +2177,30 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>DEROEUX</t>
+          <t>HERLEMONT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Aaron</t>
+          <t>Maxime</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9:56</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
@@ -2168,30 +2208,30 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>WYCKAERT</t>
+          <t>DREANO-LENGLET</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Nicolas</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9:57</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -2199,7 +2239,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ROCHE</t>
+          <t>BRUNIAUX</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -2208,21 +2248,21 @@
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -2230,30 +2270,30 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>DEVAUCHELLE</t>
+          <t>DELABRE</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Tyméo</t>
+          <t>Florimond</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:31</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -2261,30 +2301,30 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>DESFRANCOIS</t>
+          <t>CAUCHY</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:48</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
@@ -2292,30 +2332,30 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>LAMOUR</t>
+          <t>LELEUX</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:53</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -2323,30 +2363,30 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ROUGEGREZ</t>
+          <t>CLAY</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Mael</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10:56</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>4ème</t>
+          <t>2nde Pro Gaïa</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -2354,30 +2394,30 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>GELE</t>
+          <t>GUILBERT</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Yanis</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11:05</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -2385,30 +2425,30 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>GRONNIER</t>
+          <t>BERTHE</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Matéo</t>
+          <t>Charles</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>8:49</t>
+          <t>8:38</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
@@ -2416,30 +2456,30 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>DUFRANNE</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Léopold</t>
+          <t>Benjamin</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>9:53</t>
+          <t>9:20</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
@@ -2447,30 +2487,30 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>PIETRZAK</t>
+          <t>BONEL</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Eden</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>9:41</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
@@ -2478,30 +2518,30 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>BELLIARD</t>
+          <t>DESSENNE</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Julien</t>
+          <t>Adrien</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:50</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
@@ -2509,30 +2549,30 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>LESAFFRE</t>
+          <t>DUPONT</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Alexandre</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>10:42</t>
+          <t>10:54</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
@@ -2540,30 +2580,30 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>DESCAMPS</t>
+          <t>LEIGNEL</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Jeanne</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>11:53</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
@@ -2571,30 +2611,30 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>PIOLE</t>
+          <t>WINTREBERT</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Jean</t>
+          <t>Marion</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>10:47</t>
+          <t>13:04</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>1ère STAV</t>
+          <t>2nde Mendel</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
@@ -2602,30 +2642,30 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>CARON</t>
+          <t>DEGARDIN</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>13:14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
@@ -2633,30 +2673,30 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>HERLEMONT</t>
+          <t>ROUSSEL</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Maxime</t>
+          <t>Vivien</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>9:56</t>
+          <t>9:40</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
@@ -2664,30 +2704,30 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>DREANO-LENGLET</t>
+          <t>LAVISSE</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Nicolas</t>
+          <t>Paul-Edouard</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>9:57</t>
+          <t>9:55</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
@@ -2695,30 +2735,30 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>BRUNIAUX</t>
+          <t>BRIANCHON</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Timothé</t>
+          <t>Evan</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>10:12</t>
+          <t>10:27</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -2726,30 +2766,30 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>DELABRE</t>
+          <t>DEGENNE</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Florimond</t>
+          <t>Valentin</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>10:31</t>
+          <t>10:46</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
@@ -2757,30 +2797,30 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>CAUCHY</t>
+          <t>VICTORIA</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>10:48</t>
+          <t>11:06</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
@@ -2788,30 +2828,30 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>LELEUX</t>
+          <t>HADENGUE</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Alban</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>10:53</t>
+          <t>11:11</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
@@ -2819,30 +2859,30 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>CLAY</t>
+          <t>BONNEVAL</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>11:40</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Gaïa</t>
+          <t>2nde Pro Aristée</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
@@ -2850,23 +2890,23 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>GUILBERT</t>
+          <t>LAFFINEUR</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Enzo</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>14:02</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3161,7 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
@@ -3129,30 +3169,30 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>BERTHE</t>
+          <t>LUSSIEZ</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Charles</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>8:38</t>
+          <t>10:01</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
@@ -3160,30 +3200,30 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>TEMPEZ</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Benjamin</t>
+          <t>Antoine</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>9:20</t>
+          <t>10:20</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
@@ -3191,30 +3231,30 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>BONEL</t>
+          <t>CAMUS</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Hugo</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>9:41</t>
+          <t>10:24</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
@@ -3222,30 +3262,30 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>DESSENNE</t>
+          <t>BOUTEILLER</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Adrien</t>
+          <t>Nathan</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>10:51</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
@@ -3253,30 +3293,30 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>DUPONT</t>
+          <t>BOURGOGNE</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Alexandre</t>
+          <t>Célestine</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>10:54</t>
+          <t>12:14</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
@@ -3284,30 +3324,30 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>LEIGNEL</t>
+          <t>LEVERT</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Jeanne</t>
+          <t>Quentin</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>12:21</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
@@ -3315,30 +3355,30 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>WINTREBERT</t>
+          <t>BRUNEEL</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Marion</t>
+          <t>Pierre-Vincent</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:38</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>2nde Mendel</t>
+          <t>1ère Pro</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
@@ -3346,23 +3386,23 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>DEGARDIN</t>
+          <t>FOVEAU</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Luna</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:27</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3657,7 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B58" s="4" t="n">
@@ -3625,30 +3665,30 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>VALENTIN</t>
+          <t>BOURBON</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Raphael</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>9:53</t>
+          <t>8:53</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
@@ -3656,30 +3696,30 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>GAGNON</t>
+          <t>LEIGNEL</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Madeline</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>9:53</t>
+          <t>11:01</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B60" s="4" t="n">
@@ -3687,30 +3727,30 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>CORRE</t>
+          <t>DRUET</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Maël</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>11:46</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B61" s="4" t="n">
@@ -3718,30 +3758,30 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>MERVEILLE</t>
+          <t>BRULIN</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Albéric</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:56</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B62" s="4" t="n">
@@ -3749,30 +3789,30 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>DUHAMEL</t>
+          <t>LEMAITRE</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Rémi</t>
+          <t>Lola</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:06</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B63" s="4" t="n">
@@ -3780,30 +3820,30 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>TOP</t>
+          <t>LETOURMY</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Tédy</t>
+          <t>Maximilien</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>12:41</t>
+          <t>12:20</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B64" s="4" t="n">
@@ -3811,30 +3851,30 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>ELIE</t>
+          <t>GROS</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Quantin</t>
+          <t>Léopold</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:49</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 App</t>
+          <t>2nde Pasteur</t>
         </is>
       </c>
       <c r="B65" s="4" t="n">
@@ -3842,30 +3882,30 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>DULOT</t>
+          <t>CUCHEVAL</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:16</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B66" s="4" t="n">
@@ -3873,30 +3913,30 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>ROUSSEL</t>
+          <t>DONNEZ</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Vivien</t>
+          <t>Nino</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>10:06</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
@@ -3904,30 +3944,30 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>LAVISSE</t>
+          <t>DEBUIRE</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Paul-Edouard</t>
+          <t>Victor</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>9:55</t>
+          <t>10:19</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B68" s="4" t="n">
@@ -3935,30 +3975,30 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>BRIANCHON</t>
+          <t>ROCROY</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Evan</t>
+          <t>Ethan</t>
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:22</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B69" s="4" t="n">
@@ -3966,30 +4006,30 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>DEGENNE</t>
+          <t>HACCART</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Valentin</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>10:46</t>
+          <t>11:18</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B70" s="4" t="n">
@@ -3997,30 +4037,30 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>VICTORIA</t>
+          <t>BOULET</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Léo</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>11:48</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
@@ -4028,30 +4068,30 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>HADENGUE</t>
+          <t>CARPENTIER</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Alban</t>
+          <t>Antonin</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>11:11</t>
+          <t>12:36</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B72" s="4" t="n">
@@ -4059,30 +4099,30 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>BONNEVAL</t>
+          <t>LEFEVRE COUPE</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Baptiste</t>
+          <t>Elora</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>12:37</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2nde Pro Aristée</t>
+          <t>3ème</t>
         </is>
       </c>
       <c r="B73" s="4" t="n">
@@ -4090,30 +4130,30 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>LAFFINEUR</t>
+          <t>PROBIN</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>Enzo</t>
+          <t>Tristan</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>15:15</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B74" s="4" t="n">
@@ -4121,7 +4161,7 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>LUSSIEZ</t>
+          <t>VALENTIN</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
@@ -4130,21 +4170,21 @@
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>9:53</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B75" s="4" t="n">
@@ -4152,30 +4192,30 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>TEMPEZ</t>
+          <t>GAGNON</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Antoine</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>9:53</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B76" s="4" t="n">
@@ -4183,30 +4223,30 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>CAMUS</t>
+          <t>CORRE</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Maël</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>11:23</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B77" s="4" t="n">
@@ -4214,30 +4254,30 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>BOUTEILLER</t>
+          <t>MERVEILLE</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Nathan</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>11:58</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B78" s="4" t="n">
@@ -4245,30 +4285,30 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>BOURGOGNE</t>
+          <t>DUHAMEL</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Célestine</t>
+          <t>Rémi</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:31</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B79" s="4" t="n">
@@ -4276,30 +4316,30 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>COURTOIS</t>
+          <t>TOP</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Luka</t>
+          <t>Tédy</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>13:27</t>
+          <t>12:41</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B80" s="4" t="n">
@@ -4307,30 +4347,30 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>LEVERT</t>
+          <t>ELIE</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Quentin</t>
+          <t>Quantin</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>13:00</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro</t>
+          <t>GDEA 1 App</t>
         </is>
       </c>
       <c r="B81" s="4" t="n">
@@ -4338,30 +4378,30 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>BRUNEEL</t>
+          <t>DULOT</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Pierre-Vincent</t>
+          <t>Baptiste</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>13:22</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B82" s="4" t="n">
@@ -4369,30 +4409,30 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>BOURBON</t>
+          <t>DUPONT</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Raphael</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>8:53</t>
+          <t>10:04</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B83" s="4" t="n">
@@ -4400,30 +4440,30 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>LEIGNEL</t>
+          <t>VALCKE</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Madeline</t>
+          <t>Anthime</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:32</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B84" s="4" t="n">
@@ -4431,30 +4471,30 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>DRUET</t>
+          <t>LAMIAUX</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>11:08</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B85" s="4" t="n">
@@ -4462,30 +4502,30 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>BRULIN</t>
+          <t>MILLE</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Albéric</t>
+          <t>Lubin</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>12:29</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B86" s="4" t="n">
@@ -4493,30 +4533,30 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>LEMAITRE</t>
+          <t>POLIN</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Lola</t>
+          <t>Clémentine</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>12:06</t>
+          <t>13:00</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B87" s="4" t="n">
@@ -4524,30 +4564,30 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>LETOURMY</t>
+          <t>VIARD</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Maximilien</t>
+          <t>Camille</t>
         </is>
       </c>
       <c r="E87" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>13:59</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B88" s="4" t="n">
@@ -4555,30 +4595,30 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>GROS</t>
+          <t>COPIN</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Léopold</t>
+          <t>Léontine</t>
         </is>
       </c>
       <c r="E88" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>13:59</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>2nde Pasteur</t>
+          <t>1ère G</t>
         </is>
       </c>
       <c r="B89" s="4" t="n">
@@ -4586,23 +4626,23 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>CUCHEVAL</t>
+          <t>LAVAQUERIE</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Léa</t>
         </is>
       </c>
       <c r="E89" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>13:16</t>
+          <t>14:00</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5393,7 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B114" s="4" t="n">
@@ -5361,30 +5401,30 @@
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>DUPONT</t>
+          <t>DERUIT</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Maxime</t>
         </is>
       </c>
       <c r="E114" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F114" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:37</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B115" s="4" t="n">
@@ -5392,30 +5432,30 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>VALCKE</t>
+          <t>ANSELIN</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>Anthime</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="E115" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F115" s="4" t="n">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>11:59</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B116" s="4" t="n">
@@ -5423,30 +5463,30 @@
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>LAMIAUX</t>
+          <t>CAMUS</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="E116" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F116" s="4" t="n">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>12:42</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B117" s="4" t="n">
@@ -5454,30 +5494,30 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>MILLE</t>
+          <t>COMBLE</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr">
         <is>
-          <t>Lubin</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="E117" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F117" s="4" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>13:29</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B118" s="4" t="n">
@@ -5485,30 +5525,30 @@
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>POLIN</t>
+          <t>BERTOUX</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t>Clémentine</t>
+          <t>Jules</t>
         </is>
       </c>
       <c r="E118" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F118" s="4" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:58</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B119" s="4" t="n">
@@ -5516,30 +5556,30 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>VIARD</t>
+          <t>LAGACHE</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>Camille</t>
+          <t>Mathieu</t>
         </is>
       </c>
       <c r="E119" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F119" s="4" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:58</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B120" s="4" t="n">
@@ -5547,30 +5587,30 @@
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>COPIN</t>
+          <t>DALLERY</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>Léontine</t>
+          <t>Jules</t>
         </is>
       </c>
       <c r="E120" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F120" s="4" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="G120" s="4" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>14:04</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>1ère G</t>
+          <t>1ère Pro App</t>
         </is>
       </c>
       <c r="B121" s="4" t="n">
@@ -5578,30 +5618,30 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>LAVAQUERIE</t>
+          <t>VIGNE--PLAISANT</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>Léa</t>
+          <t>Marius</t>
         </is>
       </c>
       <c r="E121" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F121" s="4" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="G121" s="4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:49</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B122" s="4" t="n">
@@ -5609,30 +5649,30 @@
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>GOSSELIN</t>
+          <t>DEROEUX</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Aaron</t>
         </is>
       </c>
       <c r="E122" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F122" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G122" s="4" t="inlineStr">
         <is>
-          <t>10:14</t>
+          <t>10:41</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B123" s="4" t="n">
@@ -5640,30 +5680,30 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>BELKHAYAT</t>
+          <t>WYCKAERT</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
         <is>
-          <t>Thibaut</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="E123" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F123" s="4" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G123" s="4" t="inlineStr">
         <is>
-          <t>10:31</t>
+          <t>10:42</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B124" s="4" t="n">
@@ -5671,30 +5711,30 @@
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>MINEZ</t>
+          <t>ROCHE</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t>Clément</t>
+          <t>Timothé</t>
         </is>
       </c>
       <c r="E124" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F124" s="4" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="G124" s="4" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:00</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B125" s="4" t="n">
@@ -5702,30 +5742,30 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>DELVA</t>
+          <t>DEVAUCHELLE</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>Simon</t>
+          <t>Tyméo</t>
         </is>
       </c>
       <c r="E125" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F125" s="4" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="G125" s="4" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>14:31</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B126" s="4" t="n">
@@ -5733,30 +5773,30 @@
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>GRIN</t>
+          <t>DESFRANCOIS</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>Louis</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="E126" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F126" s="4" t="n">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="G126" s="4" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:32</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B127" s="4" t="n">
@@ -5764,30 +5804,30 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>GENCE</t>
+          <t>LAMOUR</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>Raphaël</t>
+          <t>Hugo</t>
         </is>
       </c>
       <c r="E127" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F127" s="4" t="n">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="G127" s="4" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>14:42</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B128" s="4" t="n">
@@ -5795,30 +5835,30 @@
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>SNEESSENS</t>
+          <t>ROUGEGREZ</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr">
         <is>
-          <t>Gabriel</t>
+          <t>Mael</t>
         </is>
       </c>
       <c r="E128" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F128" s="4" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="G128" s="4" t="inlineStr">
         <is>
-          <t>16:16</t>
+          <t>15:13</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>GDEA 1 Sco</t>
+          <t>4ème</t>
         </is>
       </c>
       <c r="B129" s="4" t="n">
@@ -5826,30 +5866,30 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>DELCROIX</t>
+          <t>GELE</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>Alexis</t>
+          <t>Yanis</t>
         </is>
       </c>
       <c r="E129" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F129" s="4" t="n">
-        <v>103</v>
+        <v>15</v>
       </c>
       <c r="G129" s="4" t="inlineStr">
         <is>
-          <t>16:54</t>
+          <t>15:14</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B130" s="4" t="n">
@@ -5857,30 +5897,30 @@
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>DERUIT</t>
+          <t>GOSSELIN</t>
         </is>
       </c>
       <c r="D130" s="5" t="inlineStr">
         <is>
-          <t>Maxime</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="E130" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F130" s="4" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="G130" s="4" t="inlineStr">
         <is>
-          <t>10:37</t>
+          <t>10:14</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B131" s="4" t="n">
@@ -5888,30 +5928,30 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>ANSELIN</t>
+          <t>BELKHAYAT</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Thibaut</t>
         </is>
       </c>
       <c r="E131" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F131" s="4" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="G131" s="4" t="inlineStr">
         <is>
-          <t>11:59</t>
+          <t>10:31</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B132" s="4" t="n">
@@ -5919,30 +5959,30 @@
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>CAMUS</t>
+          <t>MINEZ</t>
         </is>
       </c>
       <c r="D132" s="5" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Clément</t>
         </is>
       </c>
       <c r="E132" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F132" s="4" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="G132" s="4" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>11:24</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B133" s="4" t="n">
@@ -5950,30 +5990,30 @@
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>DALLERY</t>
+          <t>DELVA</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>Simon</t>
         </is>
       </c>
       <c r="E133" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F133" s="4" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="G133" s="4" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>11:57</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B134" s="4" t="n">
@@ -5981,30 +6021,30 @@
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>COMBLE</t>
+          <t>GRIN</t>
         </is>
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Louis</t>
         </is>
       </c>
       <c r="E134" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F134" s="4" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G134" s="4" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>14:21</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B135" s="4" t="n">
@@ -6012,30 +6052,30 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>BERTOUX</t>
+          <t>GENCE</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>Raphaël</t>
         </is>
       </c>
       <c r="E135" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F135" s="4" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="G135" s="4" t="inlineStr">
         <is>
-          <t>13:58</t>
+          <t>15:49</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B136" s="4" t="n">
@@ -6043,30 +6083,30 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>VIGNE--PLAISANT</t>
+          <t>SNEESSENS</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
         <is>
-          <t>Marius</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="E136" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F136" s="4" t="n">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="G136" s="4" t="inlineStr">
         <is>
-          <t>14:49</t>
+          <t>16:16</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>1ère Pro App</t>
+          <t>GDEA 1 Sco</t>
         </is>
       </c>
       <c r="B137" s="4" t="n">
@@ -6074,23 +6114,23 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>LAGACHE</t>
+          <t>DELCROIX</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>Mathieu</t>
+          <t>Alexis</t>
         </is>
       </c>
       <c r="E137" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F137" s="4" t="n">
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="G137" s="4" t="inlineStr">
         <is>
-          <t>13:58</t>
+          <t>16:54</t>
         </is>
       </c>
     </row>

</xml_diff>